<commit_message>
finished core, flash, crystal oscillator, and power regulation
</commit_message>
<xml_diff>
--- a/PCB/materials.xlsx
+++ b/PCB/materials.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\joshf\Documents\Code\USB_IR_Blaster\PCB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E75EB6B7-7DAA-4A09-8512-F879C7D98642}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A4E20FE-3077-48BE-94DA-8CE92E0E62BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{FC31D8FB-3664-43EE-8E32-81502E5E38D7}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="70">
   <si>
     <t>Description</t>
   </si>
@@ -221,10 +221,34 @@
     <t>4.7 µF ±10% 10V Ceramic Capacitor X7R 0603 (1608 Metric)</t>
   </si>
   <si>
-    <t>FLASH - NOR Memory IC 128Mbit SPI - Quad I/O 133 MHz 8-SOIC</t>
-  </si>
-  <si>
-    <t>https://www.digikey.com/en/products/detail/renesas-electronics-corporation/AT25SF128A-SHB-T/10107135</t>
+    <t>FLASH - NOR Memory IC 128Mbit SPI - Quad I/O, QPI 133 MHz 8-SOIC</t>
+  </si>
+  <si>
+    <t>W25Q128JVSIQ</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/winbond-electronics/W25Q128JVSIQ/5803943</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/c-k/PTS636SM43SMTR-LFS/10071723</t>
+  </si>
+  <si>
+    <t>PTS636SM43SMTR LFS</t>
+  </si>
+  <si>
+    <t>Tactile Switch SPST-NO Top Actuated Surface Mount</t>
+  </si>
+  <si>
+    <t>Button_Switch_SMD:SW_Push_6x3.5mm</t>
+  </si>
+  <si>
+    <t>STDCRG1-12M</t>
+  </si>
+  <si>
+    <t>https://www.mouser.com/ProductDetail/ABRACON/ABM8-272-T3?qs=QpmGXVUTftEj6miOiJBMxQ%3D%3D&amp;srsltid=AfmBOoreONVOH-K9twHGfSJF-Jpo5aXiXpnElmP-T8XmVjeTsv9DHJFU</t>
+  </si>
+  <si>
+    <t>Crystals Ultra Miniature Ceramic SMD Crystal</t>
   </si>
 </sst>
 </file>
@@ -620,7 +644,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1CDCC247-279C-4A9F-A582-D4D49D3E2219}">
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="2" width="15.265625" customWidth="1"/>
@@ -865,12 +889,40 @@
         <v>58</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="114" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:8" ht="99.75" x14ac:dyDescent="0.45">
       <c r="A12" s="2" t="s">
         <v>60</v>
       </c>
+      <c r="C12" t="s">
+        <v>61</v>
+      </c>
       <c r="E12" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" ht="99.75" x14ac:dyDescent="0.45">
+      <c r="A13" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="C13" t="s">
+        <v>64</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" ht="213.75" x14ac:dyDescent="0.45">
+      <c r="A14" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="C14" t="s">
+        <v>67</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>68</v>
       </c>
     </row>
   </sheetData>

</xml_diff>